<commit_message>
Refactor: updated all Excel files and scripts to use English headers (TEAM, Round, etc.)
</commit_message>
<xml_diff>
--- a/data/premier_league_match_data_detailed.xlsx
+++ b/data/premier_league_match_data_detailed.xlsx
@@ -431,32 +431,32 @@
     <row r="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Kolejka</t>
+          <t>Round</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Drużyna</t>
+          <t>TEAM</t>
         </is>
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>Przeciwnik</t>
+          <t>Opponent</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
         <is>
-          <t>Typ</t>
+          <t>Type</t>
         </is>
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>Punkty</t>
+          <t>Points</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>Dominacja</t>
+          <t>Domination</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -466,7 +466,7 @@
       </c>
       <c r="H1" s="1" t="inlineStr">
         <is>
-          <t>xG.1</t>
+          <t>xG_Opponent</t>
         </is>
       </c>
       <c r="I1" s="1" t="inlineStr">

</xml_diff>